<commit_message>
Update des profils métier fbc8395dc7f00a0ca09563e80a43ef669f7af60a
</commit_message>
<xml_diff>
--- a/htr-strucGenerale-CDA/ig/StructureDefinition-Evenement.xlsx
+++ b/htr-strucGenerale-CDA/ig/StructureDefinition-Evenement.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="128">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-04-18T14:53:38+00:00</t>
+    <t>2025-04-22T14:34:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Évènement (acte, traitement, diagnostic, etc…) décrit dans le document.Il y a au minimum une occurrence de cet élément pour décrire l'évènement principal avec obligatoirement une date de début et un exécutant.</t>
+    <t>Évènement (acte, traitement, diagnostic, etc…) décrit dans le document. Il y a au minimum une occurrence de cet élément pour décrire l'évènement principal avec obligatoirement une date de début et un exécutant.</t>
   </si>
   <si>
     <t>Purpose</t>
@@ -257,7 +257,12 @@
 </t>
   </si>
   <si>
-    <t>Identifiant de l’évènement documenté .</t>
+    <t>Identifiant de l’évènement documenté. 
+ Obligatoire pour :
+  - une demande d'acte d'imagerie pour porter l'Order Placer Number.
+  - un CR d’imagerie pour porter le studyInstanceUID.
+ Fourni si connu pour :
+  - une prescription pour porter l'identifiant EPU de la prescription.</t>
   </si>
   <si>
     <t>Evenement.codeEvenement</t>
@@ -267,7 +272,12 @@
 </t>
   </si>
   <si>
-    <t>Code de l’évènement documenté (obligatoire pour une Demande d'actes d'imagerie, un CR d’imagerie, CR d’examen de l’enfant et un document d’expression personnelle du patient/usager).</t>
+    <t>Code de l’évènement documenté.  
+ Obligatoire pour :
+  - une demande d'actes d'imagerie (code LOINC ='55115-0' 'Demande d’actes d’imagerie')
+  - un CR d’imagerie (code LOINC de l'acte d'imagerie),
+  - un CR d’examen de l’enfant (code SNOMED CT ='11429006' 'consultation'),
+  - un document d’expression personnelle du patient/usager (code TRE_A00 'EXP_PATIENT' 'Expression personnelle du patient').</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
@@ -366,7 +376,12 @@
     <t>Evenement.codeEvenement.translation</t>
   </si>
   <si>
-    <t>Translation (obligatoire pour un CR d’imagerie et un CR d’examen de l’enfant).</t>
+    <t>Translation. 
+ Obligatoire pour : 
+  - un CR d’imagerie pour indiquer
+   - 1..* la (ou les) modalité(s) d'acquisition,
+   - 1..* la (ou les) région(s) anatomique(s)
+  - un CR d’examen de l’enfant pour indiquer l'examen (jdv-examen-enfant-obligatoire-cisis).</t>
   </si>
   <si>
     <t>Evenement.dateHeureEvenement</t>
@@ -376,7 +391,8 @@
 </t>
   </si>
   <si>
-    <t>Date et heure de l’évènement documenté.</t>
+    <t>Date et heure de début et de fin de l’évènement documenté. 
+  Date de début obligatoire pour l'évènement documenté principal.</t>
   </si>
   <si>
     <t>Evenement.executantEvenement</t>
@@ -386,7 +402,8 @@
 </t>
   </si>
   <si>
-    <t>Exécutant.</t>
+    <t>Exécutant. 
+  Obligatoire pour l'évènement documenté principal.</t>
   </si>
   <si>
     <t>Evenement.executantEvenement.roleFonctionnel</t>
@@ -406,6 +423,10 @@
   <si>
     <t xml:space="preserve">https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/PersonneStructure
 </t>
+  </si>
+  <si>
+    <t>Exécutant. 
+  Le cadre d'exercice est obligatoire pour l'évènement documenté principal.</t>
   </si>
 </sst>
 </file>
@@ -1778,7 +1799,7 @@
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G11" t="s" s="2">
         <v>73</v>
@@ -1853,7 +1874,7 @@
         <v>118</v>
       </c>
       <c r="AG11" t="s" s="2">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="AH11" t="s" s="2">
         <v>73</v>
@@ -2096,10 +2117,10 @@
         <v>126</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>

</xml_diff>